<commit_message>
Restore third circle line with optional lid QR
</commit_message>
<xml_diff>
--- a/label_input_template.xlsx
+++ b/label_input_template.xlsx
@@ -433,7 +433,7 @@
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
@@ -508,7 +508,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>(Optional) Secondary info</t>
+          <t>(Optional)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -560,7 +560,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>(Optional) Secondary info</t>
+          <t>(Optional)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -634,7 +634,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CircleLine1, CircleLine2MainInfo, CircleLine3 become the three circle lines.</t>
+          <t>CircleLine1, CircleLine2MainInfo, and CircleLine3 can become the three circle/lid text lines. If lid QR is enabled, CircleLine3 is reserved for the QR and is not printed as text.</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UniqueID is optional. If filled and QR/barcode output is enabled, it can be encoded on the label.</t>
+          <t>UniqueID is optional. When provided, it is always encoded first because it is the safest database identifier. If it is absent, QR output can still encode descriptive label information up to the configured character limit.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace QR codes with compact Data Matrix codes
</commit_message>
<xml_diff>
--- a/label_input_template.xlsx
+++ b/label_input_template.xlsx
@@ -543,7 +543,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>IT000001</t>
+          <t>IT-HC000001</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>IT000002</t>
+          <t>IT-HC000002</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CircleLine1, CircleLine2MainInfo, and CircleLine3 can become the three circle/lid text lines. If lid QR is enabled, CircleLine3 is reserved for the QR and is not printed as text.</t>
+          <t>CircleLine1, CircleLine2MainInfo, and CircleLine3 can become the three circle/lid text lines. If lid Data Matrix is enabled, CircleLine3 is reserved for the Data Matrix and is not printed as text.</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UniqueID is optional. When provided, it is always encoded first because it is the safest database identifier. If it is absent, QR output can still encode descriptive label information up to the configured character limit.</t>
+          <t>UniqueID is optional. When provided, it is always encoded first because it is the safest database identifier. If it is absent, Data Matrix output can still encode the available circle/lid information up to the configured character limit.</t>
         </is>
       </c>
     </row>

</xml_diff>